<commit_message>
docs: save final verified E2E test report
</commit_message>
<xml_diff>
--- a/E2E_Test_Report.xlsx
+++ b/E2E_Test_Report.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>June 19, 2026  10:29</t>
+          <t>June 19, 2026  10:34</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B25" s="14" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C25" s="15" t="n">
         <v>1000</v>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="H2" s="21" t="n">
-        <v>1084</v>
+        <v>948</v>
       </c>
     </row>
     <row r="3">
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="H4" s="21" t="n">
-        <v>1561</v>
+        <v>1583</v>
       </c>
     </row>
     <row r="5">
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="H5" s="22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="H6" s="21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="H7" s="22" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="H8" s="21" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="H9" s="22" t="n">
-        <v>556</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10">
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="H10" s="21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="H11" s="22" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="H13" s="22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="H14" s="21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="H15" s="22" t="n">
-        <v>452</v>
+        <v>501</v>
       </c>
     </row>
     <row r="16">
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="H16" s="21" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="H17" s="22" t="n">
-        <v>59</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18">
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="H18" s="21" t="n">
-        <v>1561</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="19">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="H19" s="22" t="n">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="20">
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="H20" s="21" t="n">
-        <v>542</v>
+        <v>553</v>
       </c>
     </row>
     <row r="21">
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="H21" s="22" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22">
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="H23" s="22" t="n">
-        <v>461</v>
+        <v>456</v>
       </c>
     </row>
     <row r="24">
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="H25" s="22" t="n">
-        <v>1049</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="26">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="H26" s="21" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27">
@@ -2059,7 +2059,7 @@
         </is>
       </c>
       <c r="H27" s="22" t="n">
-        <v>1982</v>
+        <v>1977</v>
       </c>
     </row>
     <row r="28">
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="H30" s="21" t="n">
-        <v>1023</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="31">
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="H31" s="22" t="n">
-        <v>1955</v>
+        <v>1941</v>
       </c>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
fix: resolve Jest testing failure by ignoring selenium-tests, and update E2E test report
</commit_message>
<xml_diff>
--- a/E2E_Test_Report.xlsx
+++ b/E2E_Test_Report.xlsx
@@ -617,7 +617,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>June 19, 2026  10:34</t>
+          <t>July 03, 2026  09:55</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
         </is>
       </c>
       <c r="B24" s="14" t="n">
-        <v>57</v>
+        <v>135</v>
       </c>
       <c r="C24" s="15" t="n">
         <v>500</v>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B25" s="14" t="n">
-        <v>98</v>
+        <v>138</v>
       </c>
       <c r="C25" s="15" t="n">
         <v>1000</v>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="H2" s="21" t="n">
-        <v>948</v>
+        <v>2682</v>
       </c>
     </row>
     <row r="3">
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="H3" s="22" t="n">
-        <v>4</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4">
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="H4" s="21" t="n">
-        <v>1583</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="5">
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="H5" s="22" t="n">
-        <v>8</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="H6" s="21" t="n">
-        <v>9</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7">
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="H7" s="22" t="n">
-        <v>8</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="H8" s="21" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9">
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="H9" s="22" t="n">
-        <v>562</v>
+        <v>891</v>
       </c>
     </row>
     <row r="10">
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="H10" s="21" t="n">
-        <v>7</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11">
@@ -1419,7 +1419,7 @@
         </is>
       </c>
       <c r="H11" s="22" t="n">
-        <v>6</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12">
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="H12" s="21" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="H13" s="22" t="n">
-        <v>8</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14">
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="H14" s="21" t="n">
-        <v>7</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15">
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="H15" s="22" t="n">
-        <v>501</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="16">
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="H16" s="21" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17">
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="H17" s="22" t="n">
-        <v>82</v>
+        <v>418</v>
       </c>
     </row>
     <row r="18">
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="H18" s="21" t="n">
-        <v>1589</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="19">
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="H19" s="22" t="n">
-        <v>548</v>
+        <v>721</v>
       </c>
     </row>
     <row r="20">
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="H20" s="21" t="n">
-        <v>553</v>
+        <v>751</v>
       </c>
     </row>
     <row r="21">
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="H21" s="22" t="n">
-        <v>54</v>
+        <v>642</v>
       </c>
     </row>
     <row r="22">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="H22" s="21" t="n">
-        <v>8</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23">
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="H23" s="22" t="n">
-        <v>456</v>
+        <v>746</v>
       </c>
     </row>
     <row r="24">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="H24" s="21" t="n">
-        <v>6</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25">
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="H25" s="22" t="n">
-        <v>1046</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="26">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="H26" s="21" t="n">
-        <v>8</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27">
@@ -2059,7 +2059,7 @@
         </is>
       </c>
       <c r="H27" s="22" t="n">
-        <v>1977</v>
+        <v>3126</v>
       </c>
     </row>
     <row r="28">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H28" s="21" t="n">
-        <v>10</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29">
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="H29" s="22" t="n">
-        <v>7</v>
+        <v>41</v>
       </c>
     </row>
     <row r="30">
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="H30" s="21" t="n">
-        <v>1021</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="31">
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="H31" s="22" t="n">
-        <v>1941</v>
+        <v>2740</v>
       </c>
     </row>
     <row r="32">

</xml_diff>